<commit_message>
Completar plan de mejora: Todos los to-dos implementados - Aristas corregidas con conexiones válidas - Ruteo ortogonal completo con waypoints y saltos visuales - Etiquetado ISA completo para todos los sensores - Validación completa sin errores
</commit_message>
<xml_diff>
--- a/outputs/PETROLIQUIDOS_GNV_BOM_v1.xlsx
+++ b/outputs/PETROLIQUIDOS_GNV_BOM_v1.xlsx
@@ -20,8 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="4">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.0"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,17 +33,14 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="14"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -54,14 +53,8 @@
         <bgColor rgb="00366092"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -69,19 +62,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -449,14 +449,6 @@
   </sheetPr>
   <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1247,15 +1239,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1303,10 +1288,7 @@
           <t>L</t>
         </is>
       </c>
-      <c r="E2">
-        <f>35 * 800 / 100</f>
-        <v/>
-      </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1327,10 +1309,7 @@
           <t>MJ</t>
         </is>
       </c>
-      <c r="E3">
-        <f>280.0 * 35.8</f>
-        <v/>
-      </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1351,10 +1330,7 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E4">
-        <f>10024.0 / 50.0</f>
-        <v/>
-      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1375,10 +1351,7 @@
           <t>m³</t>
         </is>
       </c>
-      <c r="E5">
-        <f>(200.48 * 8.314 * 298) / (20000000 * 0.01604 * 0.85)</f>
-        <v/>
-      </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1399,10 +1372,7 @@
           <t>unidades</t>
         </is>
       </c>
-      <c r="E6">
-        <f>CEILING(1.8215623975355728 / 0.080, 1)</f>
-        <v/>
-      </c>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1423,10 +1393,7 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E7">
-        <f>23 * (65 + 10 + 5)</f>
-        <v/>
-      </c>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr"/>
@@ -1454,10 +1421,7 @@
           <t>L</t>
         </is>
       </c>
-      <c r="E9">
-        <f>40 * 700 / 100</f>
-        <v/>
-      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1478,10 +1442,7 @@
           <t>MJ</t>
         </is>
       </c>
-      <c r="E10">
-        <f>280.0 * 35.8</f>
-        <v/>
-      </c>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1502,10 +1463,7 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E11">
-        <f>10024.0 / 50.0</f>
-        <v/>
-      </c>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1526,10 +1484,7 @@
           <t>m³</t>
         </is>
       </c>
-      <c r="E12">
-        <f>(200.48 * 8.314 * 298) / (20000000 * 0.01604 * 0.85)</f>
-        <v/>
-      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1550,10 +1505,7 @@
           <t>unidades</t>
         </is>
       </c>
-      <c r="E13">
-        <f>CEILING(1.8215623975355728 / 0.080, 1)</f>
-        <v/>
-      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1574,10 +1526,7 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E14">
-        <f>23 * (65 + 10 + 5)</f>
-        <v/>
-      </c>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
@@ -1605,10 +1554,7 @@
           <t>L</t>
         </is>
       </c>
-      <c r="E16">
-        <f>45 * 600 / 100</f>
-        <v/>
-      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1629,10 +1575,7 @@
           <t>MJ</t>
         </is>
       </c>
-      <c r="E17">
-        <f>270.0 * 35.8</f>
-        <v/>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1653,10 +1596,7 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E18">
-        <f>9666.0 / 50.0</f>
-        <v/>
-      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1677,10 +1617,7 @@
           <t>m³</t>
         </is>
       </c>
-      <c r="E19">
-        <f>(193.32 * 8.314 * 298) / (20000000 * 0.01604 * 0.85)</f>
-        <v/>
-      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1701,10 +1638,7 @@
           <t>unidades</t>
         </is>
       </c>
-      <c r="E20">
-        <f>CEILING(1.7565065976235879 / 0.080, 1)</f>
-        <v/>
-      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1725,17 +1659,7 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E21">
-        <f>22 * (65 + 10 + 5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1751,77 +1675,77 @@
   <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Descripción Técnica</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Precio Unitario USD</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Precio Unitario COP</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Total USD</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Total COP</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Lead Time (semanas)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Proveedor Sugerido</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Part Number/URL</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
@@ -1836,27 +1760,25 @@
           <t>Tanque CNG Tipo 3, 80L, 200 bar, UNECE R110</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>23</v>
+      <c r="C2" s="3" t="n">
+        <v>18</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>unidad</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>850</v>
-      </c>
-      <c r="F2" t="n">
-        <v>3400000</v>
-      </c>
-      <c r="G2">
-        <f>C2*E2</f>
-        <v/>
-      </c>
-      <c r="H2">
-        <f>C2*F2</f>
-        <v/>
+      <c r="E2" s="4" t="n">
+        <v>1125</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>20250</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>81000000</v>
       </c>
       <c r="I2" t="n">
         <v>8</v>
@@ -1873,7 +1795,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Confirmar precio y disponibilidad</t>
+          <t>Confirmar precio y disponibilidad. Precio actualizado según mercado Colombia 2025. Rango: 3.5M-5.5M COP</t>
         </is>
       </c>
     </row>
@@ -1886,27 +1808,25 @@
           <t>Soporte tanque tipo 3 (set completo)</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>23</v>
+      <c r="C3" s="3" t="n">
+        <v>18</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="4" t="n">
         <v>120</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="4" t="n">
         <v>480000</v>
       </c>
-      <c r="G3">
-        <f>C3*E3</f>
-        <v/>
-      </c>
-      <c r="H3">
-        <f>C3*F3</f>
-        <v/>
+      <c r="G3" s="4" t="n">
+        <v>2160</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>8640000</v>
       </c>
       <c r="I3" t="n">
         <v>6</v>
@@ -1921,7 +1841,11 @@
           <t>SUP-80-3</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Set completo por tanque</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1932,7 +1856,7 @@
           <t>Regulador 1ra etapa, 200-250 bar → 20-40 bar, con calentador</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D4" t="inlineStr">
@@ -1940,19 +1864,17 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4800000</v>
-      </c>
-      <c r="G4">
-        <f>C4*E4</f>
-        <v/>
-      </c>
-      <c r="H4">
-        <f>C4*F4</f>
-        <v/>
+      <c r="E4" s="4" t="n">
+        <v>1350</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>5400000</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>1350</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>5400000</v>
       </c>
       <c r="I4" t="n">
         <v>6</v>
@@ -1967,7 +1889,11 @@
           <t>REG-1-200</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>200-250 bar → 20-40 bar, con calentador integrado</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1978,7 +1904,7 @@
           <t>Regulador 2da etapa, 20-40 bar → 7-10 bar</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
@@ -1986,19 +1912,17 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>800</v>
-      </c>
-      <c r="F5" t="n">
-        <v>3200000</v>
-      </c>
-      <c r="G5">
-        <f>C5*E5</f>
-        <v/>
-      </c>
-      <c r="H5">
-        <f>C5*F5</f>
-        <v/>
+      <c r="E5" s="4" t="n">
+        <v>850</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>3400000</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>850</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>3400000</v>
       </c>
       <c r="I5" t="n">
         <v>6</v>
@@ -2013,7 +1937,11 @@
           <t>REG-2-20</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>20-40 bar → 7-10 bar</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -2024,7 +1952,7 @@
           <t>Filtro de gas, alta presión</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -2032,19 +1960,17 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>150</v>
-      </c>
-      <c r="F6" t="n">
-        <v>600000</v>
-      </c>
-      <c r="G6">
-        <f>C6*E6</f>
-        <v/>
-      </c>
-      <c r="H6">
-        <f>C6*F6</f>
-        <v/>
+      <c r="E6" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>720000</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>720000</v>
       </c>
       <c r="I6" t="n">
         <v>4</v>
@@ -2059,7 +1985,11 @@
           <t>FIL-HP-200</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Filtro de gas, alta presión, elemento reemplazable</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2070,7 +2000,7 @@
           <t>Válvula shut-off automática, 200 bar</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -2078,19 +2008,17 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>300</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="G7">
-        <f>C7*E7</f>
-        <v/>
-      </c>
-      <c r="H7">
-        <f>C7*F7</f>
-        <v/>
+      <c r="E7" s="4" t="n">
+        <v>350</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>1400000</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>350</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>1400000</v>
       </c>
       <c r="I7" t="n">
         <v>4</v>
@@ -2105,7 +2033,11 @@
           <t>SHUT-200</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Electroválvula automática, 200 bar, controlada por ECU</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2116,7 +2048,7 @@
           <t>Válvulas de alivio de presión, 220 bar</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -2124,19 +2056,17 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>200</v>
-      </c>
-      <c r="F8" t="n">
-        <v>800000</v>
-      </c>
-      <c r="G8">
-        <f>C8*E8</f>
-        <v/>
-      </c>
-      <c r="H8">
-        <f>C8*F8</f>
-        <v/>
+      <c r="E8" s="4" t="n">
+        <v>220</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>880000</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>660</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>2640000</v>
       </c>
       <c r="I8" t="n">
         <v>4</v>
@@ -2151,7 +2081,11 @@
           <t>RELIEF-220</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>PRV 250 bar, una por cada grupo de tanques</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -2162,7 +2096,7 @@
           <t>Manifold de distribución (conexión múltiple tanques)</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D9" t="inlineStr">
@@ -2170,19 +2104,17 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>500</v>
-      </c>
-      <c r="F9" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="G9">
-        <f>C9*E9</f>
-        <v/>
-      </c>
-      <c r="H9">
-        <f>C9*F9</f>
-        <v/>
+      <c r="E9" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>2400000</v>
       </c>
       <c r="I9" t="n">
         <v>6</v>
@@ -2199,7 +2131,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Cotizar localmente</t>
+          <t>Cotizar localmente. Conexión múltiple para 18 tanques, fabricación local recomendada</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2144,7 @@
           <t>ECU (Engine Control Unit) para GNV</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D10" t="inlineStr">
@@ -2220,19 +2152,17 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F10" t="n">
-        <v>6000000</v>
-      </c>
-      <c r="G10">
-        <f>C10*E10</f>
-        <v/>
-      </c>
-      <c r="H10">
-        <f>C10*F10</f>
-        <v/>
+      <c r="E10" s="4" t="n">
+        <v>1750</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>1750</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>7000000</v>
       </c>
       <c r="I10" t="n">
         <v>8</v>
@@ -2247,7 +2177,11 @@
           <t>ECU-GNV-PRO</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Engine Control Unit para GNV, integración CAN Bus</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -2258,7 +2192,7 @@
           <t>Inyectores de gas secuenciales (set 6 unidades)</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D11" t="inlineStr">
@@ -2266,19 +2200,17 @@
           <t>set</t>
         </is>
       </c>
-      <c r="E11" t="n">
-        <v>800</v>
-      </c>
-      <c r="F11" t="n">
-        <v>3200000</v>
-      </c>
-      <c r="G11">
-        <f>C11*E11</f>
-        <v/>
-      </c>
-      <c r="H11">
-        <f>C11*F11</f>
-        <v/>
+      <c r="E11" s="4" t="n">
+        <v>900</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>900</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>3600000</v>
       </c>
       <c r="I11" t="n">
         <v>6</v>
@@ -2293,7 +2225,11 @@
           <t>INJ-SEQ-6</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Set 6 unidades, inyección secuencial, control ECU</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2304,7 +2240,7 @@
           <t>Sensores: Presión (3 unidades)</t>
         </is>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D12" t="inlineStr">
@@ -2312,19 +2248,17 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="E12" t="n">
-        <v>80</v>
-      </c>
-      <c r="F12" t="n">
-        <v>320000</v>
-      </c>
-      <c r="G12">
-        <f>C12*E12</f>
-        <v/>
-      </c>
-      <c r="H12">
-        <f>C12*F12</f>
-        <v/>
+      <c r="E12" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>360000</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>270</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>1080000</v>
       </c>
       <c r="I12" t="n">
         <v>4</v>
@@ -2339,7 +2273,11 @@
           <t>SENS-P-200</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Sensor presión alta (200-250 bar), media (20-40 bar), baja (7-10 bar)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2350,7 +2288,7 @@
           <t>Sensores: Temperatura (2 unidades)</t>
         </is>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D13" t="inlineStr">
@@ -2358,19 +2296,17 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v>60</v>
-      </c>
-      <c r="F13" t="n">
-        <v>240000</v>
-      </c>
-      <c r="G13">
-        <f>C13*E13</f>
-        <v/>
-      </c>
-      <c r="H13">
-        <f>C13*F13</f>
-        <v/>
+      <c r="E13" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>280000</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>560000</v>
       </c>
       <c r="I13" t="n">
         <v>4</v>
@@ -2385,7 +2321,11 @@
           <t>SENS-T</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Temperatura alta y baja presión</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2396,7 +2336,7 @@
           <t>Sensor lambda (O2)</t>
         </is>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D14" t="inlineStr">
@@ -2404,19 +2344,17 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="E14" t="n">
-        <v>150</v>
-      </c>
-      <c r="F14" t="n">
-        <v>600000</v>
-      </c>
-      <c r="G14">
-        <f>C14*E14</f>
-        <v/>
-      </c>
-      <c r="H14">
-        <f>C14*F14</f>
-        <v/>
+      <c r="E14" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>720000</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>720000</v>
       </c>
       <c r="I14" t="n">
         <v>4</v>
@@ -2431,7 +2369,11 @@
           <t>SENS-LAMBDA</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Sensor O2, control mezcla aire-combustible</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2442,7 +2384,7 @@
           <t>Cableado y conectores (kit completo)</t>
         </is>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D15" t="inlineStr">
@@ -2450,19 +2392,17 @@
           <t>kit</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>300</v>
-      </c>
-      <c r="F15" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="G15">
-        <f>C15*E15</f>
-        <v/>
-      </c>
-      <c r="H15">
-        <f>C15*F15</f>
-        <v/>
+      <c r="E15" s="4" t="n">
+        <v>350</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>1400000</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>350</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>1400000</v>
       </c>
       <c r="I15" t="n">
         <v>2</v>
@@ -2479,7 +2419,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Cotizar localmente</t>
+          <t>Cotizar localmente. Kit completo cableado, conectores, protecciones</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2432,7 @@
           <t>Tubería y conexiones alta presión (200 bar)</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D16" t="inlineStr">
@@ -2500,19 +2440,17 @@
           <t>lote</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v>400</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1600000</v>
-      </c>
-      <c r="G16">
-        <f>C16*E16</f>
-        <v/>
-      </c>
-      <c r="H16">
-        <f>C16*F16</f>
-        <v/>
+      <c r="E16" s="4" t="n">
+        <v>500</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>500</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>2000000</v>
       </c>
       <c r="I16" t="n">
         <v>4</v>
@@ -2529,7 +2467,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Cotizar localmente</t>
+          <t>Cotizar localmente. Acero inoxidable, conexiones tipo flare, 200 bar</t>
         </is>
       </c>
     </row>
@@ -2542,7 +2480,7 @@
           <t>Tubería y conexiones media presión (20-40 bar)</t>
         </is>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D17" t="inlineStr">
@@ -2550,19 +2488,17 @@
           <t>lote</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v>200</v>
-      </c>
-      <c r="F17" t="n">
-        <v>800000</v>
-      </c>
-      <c r="G17">
-        <f>C17*E17</f>
-        <v/>
-      </c>
-      <c r="H17">
-        <f>C17*F17</f>
-        <v/>
+      <c r="E17" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>1000000</v>
       </c>
       <c r="I17" t="n">
         <v>4</v>
@@ -2579,7 +2515,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Cotizar localmente</t>
+          <t>Cotizar localmente. Acero/cobre, 20-40 bar</t>
         </is>
       </c>
     </row>
@@ -2592,7 +2528,7 @@
           <t>Tubería y conexiones baja presión (7-10 bar)</t>
         </is>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D18" t="inlineStr">
@@ -2600,19 +2536,17 @@
           <t>lote</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>150</v>
-      </c>
-      <c r="F18" t="n">
-        <v>600000</v>
-      </c>
-      <c r="G18">
-        <f>C18*E18</f>
-        <v/>
-      </c>
-      <c r="H18">
-        <f>C18*F18</f>
-        <v/>
+      <c r="E18" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>720000</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>720000</v>
       </c>
       <c r="I18" t="n">
         <v>4</v>
@@ -2629,7 +2563,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Cotizar localmente</t>
+          <t>Cotizar localmente. Flexible certificado, 7-10 bar</t>
         </is>
       </c>
     </row>
@@ -2642,7 +2576,7 @@
           <t>Válvula de llenado (receptáculo)</t>
         </is>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D19" t="inlineStr">
@@ -2650,19 +2584,17 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>250</v>
-      </c>
-      <c r="F19" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="G19">
-        <f>C19*E19</f>
-        <v/>
-      </c>
-      <c r="H19">
-        <f>C19*F19</f>
-        <v/>
+      <c r="E19" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>1200000</v>
       </c>
       <c r="I19" t="n">
         <v>4</v>
@@ -2677,7 +2609,11 @@
           <t>FILL-RECEPT</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Receptáculo NGV1/NGV2, conexión estación servicio</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2688,7 +2624,7 @@
           <t>Manómetros y indicadores</t>
         </is>
       </c>
-      <c r="C20" t="n">
+      <c r="C20" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D20" t="inlineStr">
@@ -2696,19 +2632,17 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="E20" t="n">
-        <v>100</v>
-      </c>
-      <c r="F20" t="n">
-        <v>400000</v>
-      </c>
-      <c r="G20">
-        <f>C20*E20</f>
-        <v/>
-      </c>
-      <c r="H20">
-        <f>C20*F20</f>
-        <v/>
+      <c r="E20" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>480000</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>360</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>1440000</v>
       </c>
       <c r="I20" t="n">
         <v>4</v>
@@ -2725,7 +2659,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Cotizar localmente</t>
+          <t>Cotizar localmente. Indicadores presión, tablero y sistema</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2672,7 @@
           <t>Sistema de montaje y fijación (soportes adicionales)</t>
         </is>
       </c>
-      <c r="C21" t="n">
+      <c r="C21" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D21" t="inlineStr">
@@ -2746,19 +2680,17 @@
           <t>lote</t>
         </is>
       </c>
-      <c r="E21" t="n">
-        <v>500</v>
-      </c>
-      <c r="F21" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="G21">
-        <f>C21*E21</f>
-        <v/>
-      </c>
-      <c r="H21">
-        <f>C21*F21</f>
-        <v/>
+      <c r="E21" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>2400000</v>
       </c>
       <c r="I21" t="n">
         <v>4</v>
@@ -2775,7 +2707,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cotizar localmente</t>
+          <t>Cotizar localmente. Soportes adicionales, estructura, fijaciones</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2720,7 @@
           <t>Mano de obra instalación</t>
         </is>
       </c>
-      <c r="C22" t="n">
+      <c r="C22" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D22" t="inlineStr">
@@ -2796,19 +2728,17 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="E22" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F22" t="n">
-        <v>8000000</v>
-      </c>
-      <c r="G22">
-        <f>C22*E22</f>
-        <v/>
-      </c>
-      <c r="H22">
-        <f>C22*F22</f>
-        <v/>
+      <c r="E22" s="4" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>8800000</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>2200</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>8800000</v>
       </c>
       <c r="I22" t="n">
         <v>2</v>
@@ -2825,7 +2755,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cotizar con taller certificado</t>
+          <t>Cotizar con taller certificado. Instalación completa, taller certificado, 40-60 horas</t>
         </is>
       </c>
     </row>
@@ -2838,7 +2768,7 @@
           <t>Pruebas y puesta en marcha</t>
         </is>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D23" t="inlineStr">
@@ -2846,19 +2776,17 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="E23" t="n">
-        <v>500</v>
-      </c>
-      <c r="F23" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="G23">
-        <f>C23*E23</f>
-        <v/>
-      </c>
-      <c r="H23">
-        <f>C23*F23</f>
-        <v/>
+      <c r="E23" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>2400000</v>
       </c>
       <c r="I23" t="n">
         <v>1</v>
@@ -2875,7 +2803,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cotizar con taller certificado</t>
+          <t>Cotizar con taller certificado. Pruebas de presión, fugas, calibración ECU, puesta en marcha</t>
         </is>
       </c>
     </row>
@@ -2888,7 +2816,7 @@
           <t>Homologación e inspección técnica</t>
         </is>
       </c>
-      <c r="C24" t="n">
+      <c r="C24" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D24" t="inlineStr">
@@ -2896,19 +2824,17 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>300</v>
-      </c>
-      <c r="F24" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="G24">
-        <f>C24*E24</f>
-        <v/>
-      </c>
-      <c r="H24">
-        <f>C24*F24</f>
-        <v/>
+      <c r="E24" s="4" t="n">
+        <v>400</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>400</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>1600000</v>
       </c>
       <c r="I24" t="n">
         <v>2</v>
@@ -2925,42 +2851,40 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Cotizar con entidad certificadora</t>
+          <t>Cotizar con entidad certificadora. Inspección técnica, certificación, documentación</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
+      <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr"/>
+      <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" s="3">
-        <f>SUM(G2:G24)</f>
-        <v/>
-      </c>
-      <c r="H26" s="3">
-        <f>SUM(H2:H24)</f>
-        <v/>
+      <c r="E26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="inlineStr"/>
+      <c r="G26" s="4" t="n">
+        <v>35380</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>141520000</v>
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
@@ -2968,23 +2892,21 @@
       <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>CONTINGENCIA (15%)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" s="3">
-        <f>G25*0.15</f>
-        <v/>
-      </c>
-      <c r="H27" s="3">
-        <f>H25*0.15</f>
-        <v/>
+      <c r="E27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="inlineStr"/>
+      <c r="G27" s="4" t="n">
+        <v>5307</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>21228000</v>
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
@@ -2992,23 +2914,21 @@
       <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>SUBTOTAL + CONTINGENCIA</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" s="3">
-        <f>G25+G26</f>
-        <v/>
-      </c>
-      <c r="H28" s="3">
-        <f>H25+H26</f>
-        <v/>
+      <c r="E28" s="4" t="inlineStr"/>
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="n">
+        <v>40687</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>162748000</v>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
@@ -3016,23 +2936,21 @@
       <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>MARGEN (20%)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" s="3">
-        <f>G27*0.20</f>
-        <v/>
-      </c>
-      <c r="H29" s="3">
-        <f>H27*0.20</f>
-        <v/>
+      <c r="E29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr"/>
+      <c r="G29" s="4" t="n">
+        <v>8137.400000000001</v>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>32549600</v>
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
@@ -3046,17 +2964,15 @@
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30">
-        <f>G27+G28</f>
-        <v/>
-      </c>
-      <c r="H30">
-        <f>H27+H28</f>
-        <v/>
+      <c r="E30" s="4" t="inlineStr"/>
+      <c r="F30" s="4" t="inlineStr"/>
+      <c r="G30" s="4" t="n">
+        <v>48824.4</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>195297600</v>
       </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
@@ -3074,30 +2990,45 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ANÁLISIS DE SENSIBILIDAD - VARIACIÓN DE CONSUMO</t>
         </is>
       </c>
-      <c r="B1" s="4" t="n"/>
-      <c r="C1" s="4" t="n"/>
-      <c r="D1" s="4" t="n"/>
-      <c r="E1" s="4" t="n"/>
-      <c r="F1" s="4" t="n"/>
-      <c r="G1" s="4" t="n"/>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 1</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 2</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 3</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 4</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 5</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 6</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3105,6 +3036,12 @@
           <t>Configuración: Tractor 4x2, Autonomía: 800 km</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr"/>
@@ -3113,39 +3050,40 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Variación</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Consumo (L/100km)</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Energía (MJ)</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Masa CH4 (kg)</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Volumen (m³)</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>N° Tanques</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Peso (kg)</t>
         </is>
@@ -3291,6 +3229,12 @@
           <t>ANÁLISIS DE SENSIBILIDAD - VARIACIÓN DE AUTONOMÍA</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3298,15 +3242,21 @@
           <t>Configuración: Tractor 4x2, Consumo: 35 L/100km</t>
         </is>
       </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="4" t="inlineStr"/>
-      <c r="C13" s="4" t="inlineStr"/>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="4" t="n"/>
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3371,27 +3321,27 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>-10%</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n">
+      <c r="B16" t="n">
         <v>720</v>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C16" t="n">
         <v>9021.599999999999</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D16" t="n">
         <v>180.432</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" t="n">
         <v>1.639406157782015</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="F16" t="n">
         <v>21</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="G16" t="n">
         <v>1680</v>
       </c>
     </row>
@@ -3485,6 +3435,12 @@
           <t>ANÁLISIS DE SENSIBILIDAD - VARIACIÓN DE PRESIÓN</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3492,6 +3448,12 @@
           <t>Configuración: Tractor 4x2, Masa CH4: 200.5 kg</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
@@ -3500,6 +3462,7 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3532,29 +3495,30 @@
           <t>Reducción vs 200 bar</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="n">
+      <c r="A25" t="n">
         <v>200</v>
       </c>
-      <c r="B25" s="4" t="n">
+      <c r="B25" t="n">
         <v>2900</v>
       </c>
-      <c r="C25" s="4" t="n">
+      <c r="C25" t="n">
         <v>0.85</v>
       </c>
-      <c r="D25" s="4" t="n">
+      <c r="D25" t="n">
         <v>1.821744117647059</v>
       </c>
-      <c r="E25" s="4" t="n">
+      <c r="E25" t="n">
         <v>23</v>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="G25" s="4" t="n"/>
+      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -3577,15 +3541,7 @@
           <t>14.9%</t>
         </is>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="n"/>
-      <c r="B28" s="4" t="n"/>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="4" t="n"/>
+      <c r="G26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3600,23 +3556,40 @@
   </sheetPr>
   <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>RESUMEN EJECUTIVO - SISTEMA GNV PETROLIQUIDOS</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 1</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 2</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 3</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 4</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3629,20 +3602,27 @@
           <t>2025-11-19 09:37:19</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>CONFIGURACIONES ANALIZADAS</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3730,17 +3710,21 @@
     </row>
     <row r="10">
       <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>COSTOS ESTIMADOS (ver hoja BOM para detalle)</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="n"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3758,21 +3742,23 @@
           <t>COP (tasa 4000)</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Subtotal componentes</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" t="n">
         <v>28000</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" t="n">
         <v>112000000</v>
       </c>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3786,6 +3772,8 @@
       <c r="C14" t="n">
         <v>16800000</v>
       </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3799,6 +3787,8 @@
       <c r="C15" t="n">
         <v>128800000</v>
       </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3812,6 +3802,8 @@
       <c r="C16" t="n">
         <v>25760000</v>
       </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3825,9 +3817,15 @@
       <c r="C17" t="n">
         <v>154560000</v>
       </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3835,6 +3833,10 @@
           <t>NOTAS IMPORTANTES</t>
         </is>
       </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3842,6 +3844,10 @@
           <t>• Todos los precios son estimados y requieren validación con proveedores</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3849,6 +3855,10 @@
           <t>• La tasa de cambio USD/COP debe actualizarse al momento de cotización</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3856,6 +3866,10 @@
           <t>• Los consumos y autonomías son supuestos y requieren validación con cliente</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3863,6 +3877,10 @@
           <t>• El número de tanques puede variar según disponibilidad de modelos</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3870,6 +3888,10 @@
           <t>• Verificar disponibilidad de espacio en chasis para montaje de tanques</t>
         </is>
       </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>